<commit_message>
fixe logic declaration F2 V2
</commit_message>
<xml_diff>
--- a/PAMF_DIG F2 - monthly2026-07-09.xlsx
+++ b/PAMF_DIG F2 - monthly2026-07-09.xlsx
@@ -10196,7 +10196,7 @@
         <v>0.09</v>
       </c>
       <c r="N134" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -18737,7 +18737,7 @@
         <v>0.09</v>
       </c>
       <c r="N251" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>

</xml_diff>